<commit_message>
fix: Content-Plan.xlsx tách 2 sheet (khung trống + ví dụ) cho luồng dán tay Gemini
- Gemini không tạo được .xlsx → template có sheet trống để dán từ dòng 6
- Sheet 'Ví dụ (nâng mũi)' giữ dữ liệu HN/HCM tham chiếu
- README §19: bổ sung fallback Gemini (xuất bảng/CSV → dán); §7.2 mô tả 2 sheet

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Kangnam-Content-Plan.xlsx
+++ b/templates/Kangnam-Content-Plan.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Kế hoạch nội dung 3 tầng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Kế hoạch nội dung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ví dụ (nâng mũi)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,11 +51,11 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -159,21 +160,21 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -541,6 +542,351 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KẾ HOẠCH NỘI DUNG 3 TẦNG (TOF – MOF – BOF)  |  BỆNH VIỆN THẨM MỸ KANGNAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Framework: Phễu TOF → MOF → BOF theo vùng. ➤ DÁN DỮ LIỆU TỪ DÒNG 6 (giữ nguyên dòng 1–5). Xem sheet 'Ví dụ (nâng mũi)' để tham chiếu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Nguyên tắc: Hook đúng giọng vùng (HN: chuyên môn/uy tín · HCM: trend/cảm hứng/social proof) · tổng % ngân sách mỗi vùng ≈ 100% · số liệu là gợi ý khởi điểm · chưa xác minh → ⚠ Cần xác minh từ Kangnam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1"/>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Vùng</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Tầng</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Mục tiêu CD (FB)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Tệp nhắm (Targeting)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Định dạng Ads</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>% Ngân sách</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>KPI chính</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Insight / Nỗi đau</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Góc nội dung</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Hook (đúng giọng vùng)</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="5" t="n"/>
+      <c r="J19" s="5" t="n"/>
+      <c r="K19" s="5" t="n"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="5" t="n"/>
+      <c r="J20" s="5" t="n"/>
+      <c r="K20" s="5" t="n"/>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="5" t="n"/>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="5" t="n"/>
+      <c r="I21" s="5" t="n"/>
+      <c r="J21" s="5" t="n"/>
+      <c r="K21" s="5" t="n"/>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="5" t="n"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
+      <c r="K22" s="5" t="n"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
+      <c r="I23" s="5" t="n"/>
+      <c r="J23" s="5" t="n"/>
+      <c r="K23" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A3:K3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -567,14 +913,14 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Framework: Phễu TOF → MOF → BOF theo vùng. Ví dụ minh họa: dịch vụ Nâng mũi — thay Insight/Hook theo dịch vụ, giữ nguyên nguyên tắc tầng &amp; giọng vùng.</t>
+          <t>Framework: Ví dụ minh họa dịch vụ Nâng mũi — thay Insight/Hook theo dịch vụ, giữ nguyên nguyên tắc tầng &amp; giọng vùng. (Sheet tham chiếu, không sửa)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Nguyên tắc: Hook đúng giọng vùng (HN: chuyên môn/uy tín · HCM: trend/cảm hứng/social proof) · tổng % ngân sách mỗi vùng ≈ 100% · số liệu là gợi ý khởi điểm, tối ưu theo dữ liệu thật · chưa xác minh → ⚠ Cần xác minh từ Kangnam.</t>
+          <t>Nguyên tắc: Hook đúng giọng vùng (HN: chuyên môn/uy tín · HCM: trend/cảm hứng/social proof) · tổng % ngân sách mỗi vùng ≈ 100% · số liệu là gợi ý khởi điểm · chưa xác minh → ⚠ Cần xác minh từ Kangnam.</t>
         </is>
       </c>
     </row>
@@ -637,27 +983,27 @@
       </c>
     </row>
     <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>HN</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>TOF (nhận biết/ gieo niềm tin)</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Lượt xem video / Tương tác</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Nữ 28–45 HN + tỉnh lân cận (Bắc Ninh, Hưng Yên, Hải Phòng…), sở thích làm đẹp/công sở; broad + Lookalike 1–3%</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Video bác sĩ</t>
         </is>
@@ -667,28 +1013,28 @@
           <t>25%</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>CPM · ThruPlay · CTR</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Sợ chọn sai nơi/bác sĩ; coi trọng nơi uy tín</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Khẳng định chuyên môn; định vị nơi uy tín</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>• Đằng sau một dáng mũi đẹp tự nhiên, không phải may rủi
 • Chọn nơi nâng mũi quan trọng như chọn dáng mũi</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Bật rộng gom tệp warm</t>
         </is>
@@ -696,22 +1042,22 @@
     </row>
     <row r="7" ht="95" customHeight="1">
       <c r="A7" s="8" t="n"/>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>MOF (tìm hiểu, so sánh, củng cố niềm tin)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Traffic / Tin nhắn / Lead form</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Người xem video ≥25%, tương tác Page/IG 365 ngày, truy cập web</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Video chuyên sâu · carousel so sánh</t>
         </is>
@@ -721,28 +1067,28 @@
           <t>40%</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>CPL · cost/landing view</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Cần chuyên môn rõ ràng; phân vân phương pháp</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Giáo dục &amp; so sánh chuyên sâu</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>• Trước khi nâng mũi, đây là 5 câu nên hỏi thẳng bác sĩ của bạn
 • Nâng mũi cấu trúc và bán cấu trúc khác nhau như thế nào?</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Nuôi dưỡng dài, nhấn chuyên môn &amp; an toàn</t>
         </is>
@@ -750,22 +1096,22 @@
     </row>
     <row r="8" ht="95" customHeight="1">
       <c r="A8" s="9" t="n"/>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>BOF (chốt – mời tư vấn)</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Tin nhắn / Lead / Chuyển đổi</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Truy cập LP 30 ngày, lead chưa đặt lịch, người nhắn tin, Lookalike người đã đặt lịch</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Testimonial · mời đặt lịch</t>
         </is>
@@ -775,28 +1121,28 @@
           <t>35%</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Booking · show-up · CPA</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Cần an tâm trước khi quyết; tin vào kết quả thật</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Mời trải nghiệm tư vấn; bằng chứng an tâm</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>• Đặt lịch khám &amp; đo vẽ dáng mũi 1-1 cùng bác sĩ — phân tích trên chính gương mặt bạn
 • Hành trình nâng mũi tự nhiên của KH…</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Retarget mạnh, dùng ABO để kiểm soát</t>
         </is>
@@ -813,17 +1159,17 @@
           <t>TOF (nhận biết, cảm hứng)</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Lượt xem video / Tương tác</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Nữ 22–40 HCM + tỉnh (Bình Dương, Đồng Nai…), sở thích KOL beauty/thời trang/giải trí; broad</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Video biến đổi (KOC/ KOL)</t>
         </is>
@@ -833,28 +1179,28 @@
           <t>35%</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>ThruPlay · CTR · CPM</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Muốn nâng tầm nhan sắc; theo trend/ KOL</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Truyền cảm hứng visual; bắt trend</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>• Mũi đẹp là 'chìa khóa' thay đổi cả gương mặt!
 • Dáng mũi tự nhiên đang được nhiều người yêu thích - bạn hợp dáng nào?</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Đẩy nhiều creative trend, test liên tục</t>
         </is>
@@ -867,17 +1213,17 @@
           <t>MOF (bằng chứng thật)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Traffic / Tin nhắn</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Người xem video, người tương tác, truy cập web</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Video KOC review · carousel</t>
         </is>
@@ -887,28 +1233,28 @@
           <t>30%</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>CPL · time-view</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Muốn thấy người giống mình; sợ không hợp mặt</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Review thật; cá nhân hoá nhẹ</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>• Review thật: 30 ngày sau nâng mũi tại Kangnam trông thế nào?
 • Dáng mũi nào hợp gương mặt bạn? Soi nhanh cùng bác sĩ!</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Social proof là chính</t>
         </is>
@@ -921,17 +1267,17 @@
           <t>BOF (kết quả – trải nghiệm – ưu đãi)</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Tin nhắn / Chuyển đổi</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Truy cập LP, người nhắn tin, lead chưa đặt, Lookalike người chuyển đổi, danh sách CRM</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Before–after · ưu đãi trải nghiệm</t>
         </is>
@@ -941,28 +1287,28 @@
           <t>35%</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Booking · CPA</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>Quyết khi thấy kết quả; nhạy ưu đãi</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>Bằng chứng + mời; ưu đãi giới hạn</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>• Nhìn kết quả thật của khách giống bạn — đặt lịch trải nghiệm tư vấn cùng bác sĩ
 • Ưu đãi giới hạn - chỉ 10 suất nâng mũi trong tuần này</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Có thể đẩy ưu đãi trải nghiệm; ABO</t>
         </is>

</xml_diff>